<commit_message>
Add process emissions to 49 sectors model
</commit_message>
<xml_diff>
--- a/scenarios/49sectors_exiobase/scen_cat.xlsx
+++ b/scenarios/49sectors_exiobase/scen_cat.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Readme" sheetId="1" state="visible" r:id="rId3"/>
@@ -80,6 +80,7 @@
     <definedName function="false" hidden="false" localSheetId="2" name="phase_out_oil_heat" vbProcedure="false">NZP!$C$90</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="pkm_share" vbProcedure="false">NZP!$D$112:$J$115</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="policy_change_energy_speed" vbProcedure="false">NZP!$C$181:$AZ$185</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="policy_improvement_process_emissions_efficiency" vbProcedure="false">NZP!$C$375</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="policy_to_improve_efficiency_speed" vbProcedure="false">NZP!$C$169:$AZ$173</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="p_bioe_power" vbProcedure="false">NZP!$C$18:$I$18</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="p_bioe_residues_growth" vbProcedure="false">NZP!$C$35:$I$35</definedName>
@@ -175,6 +176,7 @@
     <definedName function="false" hidden="false" localSheetId="2" name="target_year_asymptote_pop" vbProcedure="false">nzp!#ref!</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="target_year_policy_phase_out_oil_electricity" vbProcedure="false">NZP!$C$94</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="target_year_policy_phase_out_oil_heat" vbProcedure="false">NZP!$C$95</definedName>
+    <definedName function="false" hidden="false" localSheetId="2" name="target_year_process_emissions" vbProcedure="false">NZP!$C$374</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="target_year_p_growth_RES_heat" vbProcedure="false">NZP!$C$49</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="target_year_P_rr_minerals" vbProcedure="false">NZP!$B$227</definedName>
     <definedName function="false" hidden="false" localSheetId="2" name="target_year_P_urban_land_density" vbProcedure="false">NZP!$C$406</definedName>
@@ -270,6 +272,7 @@
     <definedName function="false" hidden="false" localSheetId="3" name="phase_out_oil_heat" vbProcedure="false">PINECCAT!$C$90</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="pkm_share" vbProcedure="false">PINECCAT!$D$112:$J$115</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="policy_change_energy_speed" vbProcedure="false">PINECCAT!$C$181:$AZ$185</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="policy_improvement_process_emissions_efficiency" vbProcedure="false">PINECCAT!$C$375</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="policy_to_improve_efficiency_speed" vbProcedure="false">PINECCAT!$C$169:$AZ$173</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="p_bioe_power" vbProcedure="false">PINECCAT!$C$18:$I$18</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="p_bioe_residues_growth" vbProcedure="false">PINECCAT!$C$35:$I$35</definedName>
@@ -366,6 +369,7 @@
     <definedName function="false" hidden="false" localSheetId="3" name="target_year_asymptote_pop" vbProcedure="false">nzp!#ref!</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="target_year_policy_phase_out_oil_electricity" vbProcedure="false">PINECCAT!$C$94</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="target_year_policy_phase_out_oil_heat" vbProcedure="false">PINECCAT!$C$95</definedName>
+    <definedName function="false" hidden="false" localSheetId="3" name="target_year_process_emissions" vbProcedure="false">PINECCAT!$C$374</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="target_year_p_growth_RES_heat" vbProcedure="false">PINECCAT!$C$49</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="target_year_P_rr_minerals" vbProcedure="false">PINECCAT!$B$227</definedName>
     <definedName function="false" hidden="false" localSheetId="3" name="target_year_P_urban_land_density" vbProcedure="false">PINECCAT!$C$406</definedName>
@@ -671,7 +675,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2577" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2587" uniqueCount="657">
   <si>
     <t xml:space="preserve">This excel file contains the input data to run the MEDEAS model as documented in:</t>
   </si>
@@ -2525,6 +2529,12 @@
   </si>
   <si>
     <t xml:space="preserve">Installed capacity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Policy Improvement process intensity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Improvement</t>
   </si>
   <si>
     <t xml:space="preserve">7. ENERGY IMPORTS</t>
@@ -2661,7 +2671,7 @@
     <numFmt numFmtId="176" formatCode="0.00E+00"/>
     <numFmt numFmtId="177" formatCode="#,##0"/>
   </numFmts>
-  <fonts count="47">
+  <fonts count="50">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -2969,6 +2979,29 @@
       <charset val="1"/>
     </font>
     <font>
+      <b val="true"/>
+      <sz val="13.5"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <u val="single"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Verdana"/>
@@ -3086,7 +3119,7 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF8EA9DB"/>
-        <bgColor rgb="FF73B0DD"/>
+        <bgColor rgb="FF77AFDD"/>
       </patternFill>
     </fill>
     <fill>
@@ -3181,13 +3214,13 @@
     </fill>
     <fill>
       <patternFill patternType="darkGray">
-        <fgColor rgb="FF73B0DD"/>
+        <fgColor rgb="FF77AFDD"/>
         <bgColor rgb="FF8EA9DB"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF7C8677"/>
+        <fgColor rgb="FF7C8578"/>
         <bgColor rgb="FFA7A7A7"/>
       </patternFill>
     </fill>
@@ -3259,7 +3292,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF73B0DD"/>
+        <fgColor rgb="FF77AFDD"/>
         <bgColor rgb="FF8EA9DB"/>
       </patternFill>
     </fill>
@@ -3330,7 +3363,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="76">
+  <borders count="84">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -3364,16 +3397,16 @@
     </border>
     <border diagonalUp="false" diagonalDown="false">
       <left style="thin">
-        <color rgb="FF7C8677"/>
+        <color rgb="FF7C8578"/>
       </left>
       <right style="thin">
-        <color rgb="FF7C8677"/>
+        <color rgb="FF7C8578"/>
       </right>
       <top style="thin">
-        <color rgb="FF7C8677"/>
+        <color rgb="FF7C8578"/>
       </top>
       <bottom style="thin">
-        <color rgb="FF7C8677"/>
+        <color rgb="FF7C8578"/>
       </bottom>
       <diagonal/>
     </border>
@@ -3867,7 +3900,7 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin">
-        <color rgb="FF7C8677"/>
+        <color rgb="FF7C8578"/>
       </bottom>
       <diagonal/>
     </border>
@@ -3876,6 +3909,62 @@
       <right style="medium"/>
       <top style="thin"/>
       <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thick"/>
+      <right style="medium"/>
+      <top style="thick"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="thick"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="thick"/>
+      <top style="thick"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thick"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="thick"/>
+      <top style="medium"/>
+      <bottom style="medium"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thick"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="thick"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="medium"/>
+      <bottom style="thick"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="medium"/>
+      <right style="thick"/>
+      <top style="medium"/>
+      <bottom style="thick"/>
       <diagonal/>
     </border>
     <border diagonalUp="false" diagonalDown="false">
@@ -4176,7 +4265,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="432">
+  <cellXfs count="441">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5633,6 +5722,42 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="42" fillId="44" borderId="71" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="42" fillId="44" borderId="72" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="42" fillId="44" borderId="73" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="39" borderId="74" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="45" borderId="49" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="44" fillId="46" borderId="75" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="39" borderId="76" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="43" fillId="45" borderId="77" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="43" fillId="46" borderId="78" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="23" fillId="47" borderId="31" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5641,11 +5766,11 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="45" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="43" fillId="49" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="46" fillId="49" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5665,11 +5790,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="44" fillId="46" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="47" fillId="46" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="44" fillId="46" borderId="48" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="47" fillId="46" borderId="48" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5689,19 +5814,19 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="46" fillId="50" borderId="71" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="49" fillId="50" borderId="79" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="46" fillId="50" borderId="72" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="49" fillId="50" borderId="80" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="37" fillId="3" borderId="73" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="37" fillId="3" borderId="81" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="46" fillId="51" borderId="49" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="49" fillId="51" borderId="49" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5721,7 +5846,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="46" fillId="50" borderId="49" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="49" fillId="50" borderId="49" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5797,7 +5922,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="5" borderId="74" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="5" borderId="82" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5837,7 +5962,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="43" fillId="54" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="46" fillId="54" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5877,7 +6002,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="3" borderId="75" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="27" fillId="3" borderId="83" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -6037,7 +6162,7 @@
       <rgbColor rgb="FFD9E1F2"/>
       <rgbColor rgb="FFAFD095"/>
       <rgbColor rgb="FFBFBFBF"/>
-      <rgbColor rgb="FF7C8677"/>
+      <rgbColor rgb="FF7C8578"/>
       <rgbColor rgb="FF8EA9DB"/>
       <rgbColor rgb="FFC9C9C9"/>
       <rgbColor rgb="FFFFFFCC"/>
@@ -6063,7 +6188,7 @@
       <rgbColor rgb="FFB4C6E7"/>
       <rgbColor rgb="FFFFCC99"/>
       <rgbColor rgb="FF4472C4"/>
-      <rgbColor rgb="FF73B0DD"/>
+      <rgbColor rgb="FF77AFDD"/>
       <rgbColor rgb="FFA9D18E"/>
       <rgbColor rgb="FFFFC000"/>
       <rgbColor rgb="FFFAC090"/>
@@ -34067,14 +34192,34 @@
     <row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="39"/>
     </row>
-    <row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A373" s="39"/>
+    <row r="373" customFormat="false" ht="19.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A373" s="364" t="s">
+        <v>617</v>
+      </c>
+      <c r="B373" s="365"/>
+      <c r="C373" s="366"/>
     </row>
     <row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A374" s="39"/>
+      <c r="A374" s="367" t="s">
+        <v>412</v>
+      </c>
+      <c r="B374" s="368" t="s">
+        <v>17</v>
+      </c>
+      <c r="C374" s="369" t="n">
+        <v>2050</v>
+      </c>
     </row>
     <row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A375" s="39"/>
+      <c r="A375" s="370" t="s">
+        <v>618</v>
+      </c>
+      <c r="B375" s="371" t="s">
+        <v>305</v>
+      </c>
+      <c r="C375" s="372" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="39"/>
@@ -34105,12 +34250,12 @@
     </row>
     <row r="385" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A385" s="189" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="386" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A386" s="212" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="B386" s="212"/>
       <c r="C386" s="212"/>
@@ -34122,7 +34267,7 @@
       <c r="I386" s="212"/>
     </row>
     <row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A387" s="364"/>
+      <c r="A387" s="373"/>
       <c r="B387" s="195" t="s">
         <v>17</v>
       </c>
@@ -34150,7 +34295,7 @@
     </row>
     <row r="388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A388" s="213" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="B388" s="195" t="s">
         <v>124</v>
@@ -34179,7 +34324,7 @@
     </row>
     <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="213" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B389" s="195" t="s">
         <v>124</v>
@@ -34208,7 +34353,7 @@
     </row>
     <row r="390" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A390" s="232" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="B390" s="198" t="s">
         <v>124</v>
@@ -34237,14 +34382,14 @@
     </row>
     <row r="391" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A391" s="173"/>
-      <c r="B391" s="365"/>
-      <c r="C391" s="365"/>
+      <c r="B391" s="374"/>
+      <c r="C391" s="374"/>
       <c r="D391" s="356"/>
       <c r="E391" s="39"/>
     </row>
     <row r="392" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A392" s="212" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="B392" s="212"/>
       <c r="C392" s="212"/>
@@ -34256,7 +34401,7 @@
       <c r="I392" s="212"/>
     </row>
     <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A393" s="364"/>
+      <c r="A393" s="373"/>
       <c r="B393" s="195" t="s">
         <v>17</v>
       </c>
@@ -34284,7 +34429,7 @@
     </row>
     <row r="394" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A394" s="213" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="B394" s="195" t="s">
         <v>124</v>
@@ -34313,7 +34458,7 @@
     </row>
     <row r="395" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A395" s="232" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B395" s="198" t="s">
         <v>305</v>
@@ -34342,30 +34487,30 @@
     </row>
     <row r="396" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A396" s="173"/>
-      <c r="B396" s="365"/>
-      <c r="C396" s="366"/>
+      <c r="B396" s="374"/>
+      <c r="C396" s="375"/>
       <c r="D396" s="356"/>
       <c r="E396" s="39"/>
     </row>
     <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="173"/>
-      <c r="B397" s="365"/>
-      <c r="C397" s="365"/>
+      <c r="B397" s="374"/>
+      <c r="C397" s="374"/>
       <c r="D397" s="356"/>
-      <c r="E397" s="367"/>
-      <c r="F397" s="367"/>
-      <c r="G397" s="367"/>
-      <c r="H397" s="367"/>
-      <c r="I397" s="367"/>
+      <c r="E397" s="376"/>
+      <c r="F397" s="376"/>
+      <c r="G397" s="376"/>
+      <c r="H397" s="376"/>
+      <c r="I397" s="376"/>
     </row>
     <row r="398" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="189" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="399" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A399" s="212" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="B399" s="212"/>
       <c r="C399" s="212"/>
@@ -34374,7 +34519,7 @@
     </row>
     <row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A400" s="213" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="B400" s="195" t="s">
         <v>11</v>
@@ -34385,7 +34530,7 @@
     </row>
     <row r="401" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A401" s="213" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="B401" s="195" t="s">
         <v>67</v>
@@ -34396,18 +34541,18 @@
     </row>
     <row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="213" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="B402" s="195" t="s">
-        <v>630</v>
-      </c>
-      <c r="C402" s="368" t="n">
+        <v>632</v>
+      </c>
+      <c r="C402" s="377" t="n">
         <v>0.0074</v>
       </c>
     </row>
     <row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A403" s="213" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="B403" s="195" t="s">
         <v>17</v>
@@ -34418,10 +34563,10 @@
     </row>
     <row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A404" s="213" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="B404" s="195" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C404" s="197" t="n">
         <v>185</v>
@@ -34455,39 +34600,39 @@
       </c>
       <c r="B408" s="201"/>
       <c r="C408" s="201"/>
-      <c r="F408" s="369"/>
-      <c r="G408" s="369"/>
-      <c r="H408" s="369"/>
-      <c r="I408" s="369"/>
-      <c r="J408" s="369"/>
-      <c r="K408" s="369"/>
-      <c r="L408" s="369"/>
-      <c r="M408" s="369"/>
-      <c r="N408" s="369"/>
-      <c r="O408" s="369"/>
-      <c r="P408" s="369"/>
-      <c r="Q408" s="369"/>
-      <c r="R408" s="369"/>
-      <c r="S408" s="369"/>
-      <c r="T408" s="369"/>
-      <c r="U408" s="369"/>
-      <c r="V408" s="369"/>
-      <c r="W408" s="369"/>
-      <c r="X408" s="369"/>
-      <c r="Y408" s="369"/>
-      <c r="Z408" s="369"/>
-      <c r="AA408" s="369"/>
-      <c r="AB408" s="369"/>
-      <c r="AC408" s="369"/>
-      <c r="AD408" s="369"/>
-      <c r="AE408" s="369"/>
-      <c r="AF408" s="369"/>
-      <c r="AG408" s="369"/>
-      <c r="AH408" s="369"/>
-      <c r="AI408" s="369"/>
-      <c r="AJ408" s="369"/>
-      <c r="AK408" s="369"/>
-      <c r="AL408" s="369"/>
+      <c r="F408" s="378"/>
+      <c r="G408" s="378"/>
+      <c r="H408" s="378"/>
+      <c r="I408" s="378"/>
+      <c r="J408" s="378"/>
+      <c r="K408" s="378"/>
+      <c r="L408" s="378"/>
+      <c r="M408" s="378"/>
+      <c r="N408" s="378"/>
+      <c r="O408" s="378"/>
+      <c r="P408" s="378"/>
+      <c r="Q408" s="378"/>
+      <c r="R408" s="378"/>
+      <c r="S408" s="378"/>
+      <c r="T408" s="378"/>
+      <c r="U408" s="378"/>
+      <c r="V408" s="378"/>
+      <c r="W408" s="378"/>
+      <c r="X408" s="378"/>
+      <c r="Y408" s="378"/>
+      <c r="Z408" s="378"/>
+      <c r="AA408" s="378"/>
+      <c r="AB408" s="378"/>
+      <c r="AC408" s="378"/>
+      <c r="AD408" s="378"/>
+      <c r="AE408" s="378"/>
+      <c r="AF408" s="378"/>
+      <c r="AG408" s="378"/>
+      <c r="AH408" s="378"/>
+      <c r="AI408" s="378"/>
+      <c r="AJ408" s="378"/>
+      <c r="AK408" s="378"/>
+      <c r="AL408" s="378"/>
     </row>
     <row r="409" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A409" s="227" t="s">
@@ -34496,42 +34641,42 @@
       <c r="B409" s="228" t="s">
         <v>49</v>
       </c>
-      <c r="C409" s="370" t="n">
+      <c r="C409" s="379" t="n">
         <v>235</v>
       </c>
-      <c r="F409" s="369"/>
-      <c r="G409" s="369"/>
-      <c r="H409" s="369"/>
-      <c r="I409" s="369"/>
-      <c r="J409" s="369"/>
-      <c r="K409" s="369"/>
-      <c r="L409" s="369"/>
-      <c r="M409" s="369"/>
-      <c r="N409" s="369"/>
-      <c r="O409" s="369"/>
-      <c r="P409" s="369"/>
-      <c r="Q409" s="369"/>
-      <c r="R409" s="369"/>
-      <c r="S409" s="369"/>
-      <c r="T409" s="369"/>
-      <c r="U409" s="369"/>
-      <c r="V409" s="369"/>
-      <c r="W409" s="369"/>
-      <c r="X409" s="369"/>
-      <c r="Y409" s="369"/>
-      <c r="Z409" s="369"/>
-      <c r="AA409" s="369"/>
-      <c r="AB409" s="369"/>
-      <c r="AC409" s="369"/>
-      <c r="AD409" s="369"/>
-      <c r="AE409" s="369"/>
-      <c r="AF409" s="369"/>
-      <c r="AG409" s="369"/>
-      <c r="AH409" s="369"/>
-      <c r="AI409" s="369"/>
-      <c r="AJ409" s="369"/>
-      <c r="AK409" s="369"/>
-      <c r="AL409" s="369"/>
+      <c r="F409" s="378"/>
+      <c r="G409" s="378"/>
+      <c r="H409" s="378"/>
+      <c r="I409" s="378"/>
+      <c r="J409" s="378"/>
+      <c r="K409" s="378"/>
+      <c r="L409" s="378"/>
+      <c r="M409" s="378"/>
+      <c r="N409" s="378"/>
+      <c r="O409" s="378"/>
+      <c r="P409" s="378"/>
+      <c r="Q409" s="378"/>
+      <c r="R409" s="378"/>
+      <c r="S409" s="378"/>
+      <c r="T409" s="378"/>
+      <c r="U409" s="378"/>
+      <c r="V409" s="378"/>
+      <c r="W409" s="378"/>
+      <c r="X409" s="378"/>
+      <c r="Y409" s="378"/>
+      <c r="Z409" s="378"/>
+      <c r="AA409" s="378"/>
+      <c r="AB409" s="378"/>
+      <c r="AC409" s="378"/>
+      <c r="AD409" s="378"/>
+      <c r="AE409" s="378"/>
+      <c r="AF409" s="378"/>
+      <c r="AG409" s="378"/>
+      <c r="AH409" s="378"/>
+      <c r="AI409" s="378"/>
+      <c r="AJ409" s="378"/>
+      <c r="AK409" s="378"/>
+      <c r="AL409" s="378"/>
     </row>
     <row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="213" t="s">
@@ -34543,39 +34688,39 @@
       <c r="C410" s="197" t="n">
         <v>0.2</v>
       </c>
-      <c r="F410" s="369"/>
-      <c r="G410" s="369"/>
-      <c r="H410" s="369"/>
-      <c r="I410" s="369"/>
-      <c r="J410" s="369"/>
-      <c r="K410" s="369"/>
-      <c r="L410" s="369"/>
-      <c r="M410" s="369"/>
-      <c r="N410" s="369"/>
-      <c r="O410" s="369"/>
-      <c r="P410" s="369"/>
-      <c r="Q410" s="369"/>
-      <c r="R410" s="369"/>
-      <c r="S410" s="369"/>
-      <c r="T410" s="369"/>
-      <c r="U410" s="369"/>
-      <c r="V410" s="369"/>
-      <c r="W410" s="369"/>
-      <c r="X410" s="369"/>
-      <c r="Y410" s="369"/>
-      <c r="Z410" s="369"/>
-      <c r="AA410" s="369"/>
-      <c r="AB410" s="369"/>
-      <c r="AC410" s="369"/>
-      <c r="AD410" s="369"/>
-      <c r="AE410" s="369"/>
-      <c r="AF410" s="369"/>
-      <c r="AG410" s="369"/>
-      <c r="AH410" s="369"/>
-      <c r="AI410" s="369"/>
-      <c r="AJ410" s="369"/>
-      <c r="AK410" s="369"/>
-      <c r="AL410" s="369"/>
+      <c r="F410" s="378"/>
+      <c r="G410" s="378"/>
+      <c r="H410" s="378"/>
+      <c r="I410" s="378"/>
+      <c r="J410" s="378"/>
+      <c r="K410" s="378"/>
+      <c r="L410" s="378"/>
+      <c r="M410" s="378"/>
+      <c r="N410" s="378"/>
+      <c r="O410" s="378"/>
+      <c r="P410" s="378"/>
+      <c r="Q410" s="378"/>
+      <c r="R410" s="378"/>
+      <c r="S410" s="378"/>
+      <c r="T410" s="378"/>
+      <c r="U410" s="378"/>
+      <c r="V410" s="378"/>
+      <c r="W410" s="378"/>
+      <c r="X410" s="378"/>
+      <c r="Y410" s="378"/>
+      <c r="Z410" s="378"/>
+      <c r="AA410" s="378"/>
+      <c r="AB410" s="378"/>
+      <c r="AC410" s="378"/>
+      <c r="AD410" s="378"/>
+      <c r="AE410" s="378"/>
+      <c r="AF410" s="378"/>
+      <c r="AG410" s="378"/>
+      <c r="AH410" s="378"/>
+      <c r="AI410" s="378"/>
+      <c r="AJ410" s="378"/>
+      <c r="AK410" s="378"/>
+      <c r="AL410" s="378"/>
     </row>
     <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="232" t="s">
@@ -34587,39 +34732,39 @@
       <c r="C411" s="233" t="n">
         <v>2020</v>
       </c>
-      <c r="F411" s="369"/>
-      <c r="G411" s="369"/>
-      <c r="H411" s="369"/>
-      <c r="I411" s="369"/>
-      <c r="J411" s="369"/>
-      <c r="K411" s="369"/>
-      <c r="L411" s="369"/>
-      <c r="M411" s="369"/>
-      <c r="N411" s="369"/>
-      <c r="O411" s="369"/>
-      <c r="P411" s="369"/>
-      <c r="Q411" s="369"/>
-      <c r="R411" s="369"/>
-      <c r="S411" s="369"/>
-      <c r="T411" s="369"/>
-      <c r="U411" s="369"/>
-      <c r="V411" s="369"/>
-      <c r="W411" s="369"/>
-      <c r="X411" s="369"/>
-      <c r="Y411" s="369"/>
-      <c r="Z411" s="369"/>
-      <c r="AA411" s="369"/>
-      <c r="AB411" s="369"/>
-      <c r="AC411" s="369"/>
-      <c r="AD411" s="369"/>
-      <c r="AE411" s="369"/>
-      <c r="AF411" s="369"/>
-      <c r="AG411" s="369"/>
-      <c r="AH411" s="369"/>
-      <c r="AI411" s="369"/>
-      <c r="AJ411" s="369"/>
-      <c r="AK411" s="369"/>
-      <c r="AL411" s="369"/>
+      <c r="F411" s="378"/>
+      <c r="G411" s="378"/>
+      <c r="H411" s="378"/>
+      <c r="I411" s="378"/>
+      <c r="J411" s="378"/>
+      <c r="K411" s="378"/>
+      <c r="L411" s="378"/>
+      <c r="M411" s="378"/>
+      <c r="N411" s="378"/>
+      <c r="O411" s="378"/>
+      <c r="P411" s="378"/>
+      <c r="Q411" s="378"/>
+      <c r="R411" s="378"/>
+      <c r="S411" s="378"/>
+      <c r="T411" s="378"/>
+      <c r="U411" s="378"/>
+      <c r="V411" s="378"/>
+      <c r="W411" s="378"/>
+      <c r="X411" s="378"/>
+      <c r="Y411" s="378"/>
+      <c r="Z411" s="378"/>
+      <c r="AA411" s="378"/>
+      <c r="AB411" s="378"/>
+      <c r="AC411" s="378"/>
+      <c r="AD411" s="378"/>
+      <c r="AE411" s="378"/>
+      <c r="AF411" s="378"/>
+      <c r="AG411" s="378"/>
+      <c r="AH411" s="378"/>
+      <c r="AI411" s="378"/>
+      <c r="AJ411" s="378"/>
+      <c r="AK411" s="378"/>
+      <c r="AL411" s="378"/>
     </row>
     <row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A412" s="232" t="s">
@@ -34641,7 +34786,7 @@
     </row>
     <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="213" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="B415" s="195" t="s">
         <v>11</v>
@@ -34652,7 +34797,7 @@
     </row>
     <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A416" s="213" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="B416" s="195" t="s">
         <v>11</v>
@@ -34663,7 +34808,7 @@
     </row>
     <row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A417" s="213" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="B417" s="195" t="s">
         <v>11</v>
@@ -34674,12 +34819,12 @@
     </row>
     <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="232" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B418" s="198" t="s">
         <v>11</v>
       </c>
-      <c r="C418" s="371" t="n">
+      <c r="C418" s="380" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -35780,7 +35925,7 @@
       <c r="H17" s="196" t="n">
         <v>0</v>
       </c>
-      <c r="I17" s="372" t="n">
+      <c r="I17" s="381" t="n">
         <v>0</v>
       </c>
     </row>
@@ -35838,7 +35983,7 @@
       <c r="H19" s="196" t="n">
         <v>0</v>
       </c>
-      <c r="I19" s="372" t="n">
+      <c r="I19" s="381" t="n">
         <v>0</v>
       </c>
     </row>
@@ -35867,7 +36012,7 @@
       <c r="H20" s="196" t="n">
         <v>0.02058591</v>
       </c>
-      <c r="I20" s="372" t="n">
+      <c r="I20" s="381" t="n">
         <v>0.023136</v>
       </c>
     </row>
@@ -35896,7 +36041,7 @@
       <c r="H21" s="196" t="n">
         <v>0.0035</v>
       </c>
-      <c r="I21" s="372" t="n">
+      <c r="I21" s="381" t="n">
         <v>0.0035</v>
       </c>
     </row>
@@ -35925,7 +36070,7 @@
       <c r="H22" s="196" t="n">
         <v>0.028250311</v>
       </c>
-      <c r="I22" s="372" t="n">
+      <c r="I22" s="381" t="n">
         <v>0.03315265</v>
       </c>
     </row>
@@ -35954,7 +36099,7 @@
       <c r="H23" s="196" t="n">
         <v>4.999E-005</v>
       </c>
-      <c r="I23" s="372" t="n">
+      <c r="I23" s="381" t="n">
         <v>4.999E-005</v>
       </c>
     </row>
@@ -35983,7 +36128,7 @@
       <c r="H24" s="217" t="n">
         <v>0.003734</v>
       </c>
-      <c r="I24" s="373" t="n">
+      <c r="I24" s="382" t="n">
         <v>0.003734</v>
       </c>
     </row>
@@ -51421,14 +51566,34 @@
     <row r="372" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A372" s="39"/>
     </row>
-    <row r="373" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A373" s="39"/>
+    <row r="373" customFormat="false" ht="19.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A373" s="364" t="s">
+        <v>617</v>
+      </c>
+      <c r="B373" s="365"/>
+      <c r="C373" s="366"/>
     </row>
     <row r="374" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A374" s="39"/>
+      <c r="A374" s="367" t="s">
+        <v>412</v>
+      </c>
+      <c r="B374" s="368" t="s">
+        <v>17</v>
+      </c>
+      <c r="C374" s="369" t="n">
+        <v>2050</v>
+      </c>
     </row>
     <row r="375" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A375" s="39"/>
+      <c r="A375" s="370" t="s">
+        <v>618</v>
+      </c>
+      <c r="B375" s="371" t="s">
+        <v>305</v>
+      </c>
+      <c r="C375" s="372" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="376" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A376" s="39"/>
@@ -51459,12 +51624,12 @@
     </row>
     <row r="385" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A385" s="189" t="s">
-        <v>617</v>
+        <v>619</v>
       </c>
     </row>
     <row r="386" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A386" s="212" t="s">
-        <v>618</v>
+        <v>620</v>
       </c>
       <c r="B386" s="212"/>
       <c r="C386" s="212"/>
@@ -51476,7 +51641,7 @@
       <c r="I386" s="212"/>
     </row>
     <row r="387" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A387" s="364"/>
+      <c r="A387" s="373"/>
       <c r="B387" s="195" t="s">
         <v>17</v>
       </c>
@@ -51504,7 +51669,7 @@
     </row>
     <row r="388" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A388" s="213" t="s">
-        <v>619</v>
+        <v>621</v>
       </c>
       <c r="B388" s="195" t="s">
         <v>124</v>
@@ -51533,7 +51698,7 @@
     </row>
     <row r="389" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A389" s="213" t="s">
-        <v>620</v>
+        <v>622</v>
       </c>
       <c r="B389" s="195" t="s">
         <v>124</v>
@@ -51562,7 +51727,7 @@
     </row>
     <row r="390" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A390" s="232" t="s">
-        <v>621</v>
+        <v>623</v>
       </c>
       <c r="B390" s="198" t="s">
         <v>124</v>
@@ -51591,14 +51756,14 @@
     </row>
     <row r="391" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A391" s="173"/>
-      <c r="B391" s="365"/>
-      <c r="C391" s="365"/>
+      <c r="B391" s="374"/>
+      <c r="C391" s="374"/>
       <c r="D391" s="356"/>
       <c r="E391" s="39"/>
     </row>
     <row r="392" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A392" s="212" t="s">
-        <v>622</v>
+        <v>624</v>
       </c>
       <c r="B392" s="212"/>
       <c r="C392" s="212"/>
@@ -51610,7 +51775,7 @@
       <c r="I392" s="212"/>
     </row>
     <row r="393" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A393" s="364"/>
+      <c r="A393" s="373"/>
       <c r="B393" s="195" t="s">
         <v>17</v>
       </c>
@@ -51638,7 +51803,7 @@
     </row>
     <row r="394" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A394" s="213" t="s">
-        <v>623</v>
+        <v>625</v>
       </c>
       <c r="B394" s="195" t="s">
         <v>124</v>
@@ -51667,7 +51832,7 @@
     </row>
     <row r="395" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A395" s="232" t="s">
-        <v>624</v>
+        <v>626</v>
       </c>
       <c r="B395" s="198" t="s">
         <v>305</v>
@@ -51696,30 +51861,30 @@
     </row>
     <row r="396" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A396" s="173"/>
-      <c r="B396" s="365"/>
-      <c r="C396" s="366"/>
+      <c r="B396" s="374"/>
+      <c r="C396" s="375"/>
       <c r="D396" s="356"/>
       <c r="E396" s="39"/>
     </row>
     <row r="397" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A397" s="173"/>
-      <c r="B397" s="365"/>
-      <c r="C397" s="365"/>
+      <c r="B397" s="374"/>
+      <c r="C397" s="374"/>
       <c r="D397" s="356"/>
-      <c r="E397" s="367"/>
-      <c r="F397" s="367"/>
-      <c r="G397" s="367"/>
-      <c r="H397" s="367"/>
-      <c r="I397" s="367"/>
+      <c r="E397" s="376"/>
+      <c r="F397" s="376"/>
+      <c r="G397" s="376"/>
+      <c r="H397" s="376"/>
+      <c r="I397" s="376"/>
     </row>
     <row r="398" customFormat="false" ht="24.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A398" s="189" t="s">
-        <v>625</v>
+        <v>627</v>
       </c>
     </row>
     <row r="399" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A399" s="212" t="s">
-        <v>626</v>
+        <v>628</v>
       </c>
       <c r="B399" s="212"/>
       <c r="C399" s="212"/>
@@ -51728,7 +51893,7 @@
     </row>
     <row r="400" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A400" s="213" t="s">
-        <v>627</v>
+        <v>629</v>
       </c>
       <c r="B400" s="195" t="s">
         <v>11</v>
@@ -51739,7 +51904,7 @@
     </row>
     <row r="401" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A401" s="213" t="s">
-        <v>628</v>
+        <v>630</v>
       </c>
       <c r="B401" s="195" t="s">
         <v>67</v>
@@ -51750,18 +51915,18 @@
     </row>
     <row r="402" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A402" s="213" t="s">
-        <v>629</v>
+        <v>631</v>
       </c>
       <c r="B402" s="195" t="s">
-        <v>630</v>
-      </c>
-      <c r="C402" s="368" t="n">
+        <v>632</v>
+      </c>
+      <c r="C402" s="377" t="n">
         <v>0.0074</v>
       </c>
     </row>
     <row r="403" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A403" s="213" t="s">
-        <v>631</v>
+        <v>633</v>
       </c>
       <c r="B403" s="195" t="s">
         <v>17</v>
@@ -51772,10 +51937,10 @@
     </row>
     <row r="404" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A404" s="213" t="s">
-        <v>632</v>
+        <v>634</v>
       </c>
       <c r="B404" s="195" t="s">
-        <v>633</v>
+        <v>635</v>
       </c>
       <c r="C404" s="197" t="n">
         <v>185</v>
@@ -51809,39 +51974,39 @@
       </c>
       <c r="B408" s="201"/>
       <c r="C408" s="201"/>
-      <c r="F408" s="369"/>
-      <c r="G408" s="369"/>
-      <c r="H408" s="369"/>
-      <c r="I408" s="369"/>
-      <c r="J408" s="369"/>
-      <c r="K408" s="369"/>
-      <c r="L408" s="369"/>
-      <c r="M408" s="369"/>
-      <c r="N408" s="369"/>
-      <c r="O408" s="369"/>
-      <c r="P408" s="369"/>
-      <c r="Q408" s="369"/>
-      <c r="R408" s="369"/>
-      <c r="S408" s="369"/>
-      <c r="T408" s="369"/>
-      <c r="U408" s="369"/>
-      <c r="V408" s="369"/>
-      <c r="W408" s="369"/>
-      <c r="X408" s="369"/>
-      <c r="Y408" s="369"/>
-      <c r="Z408" s="369"/>
-      <c r="AA408" s="369"/>
-      <c r="AB408" s="369"/>
-      <c r="AC408" s="369"/>
-      <c r="AD408" s="369"/>
-      <c r="AE408" s="369"/>
-      <c r="AF408" s="369"/>
-      <c r="AG408" s="369"/>
-      <c r="AH408" s="369"/>
-      <c r="AI408" s="369"/>
-      <c r="AJ408" s="369"/>
-      <c r="AK408" s="369"/>
-      <c r="AL408" s="369"/>
+      <c r="F408" s="378"/>
+      <c r="G408" s="378"/>
+      <c r="H408" s="378"/>
+      <c r="I408" s="378"/>
+      <c r="J408" s="378"/>
+      <c r="K408" s="378"/>
+      <c r="L408" s="378"/>
+      <c r="M408" s="378"/>
+      <c r="N408" s="378"/>
+      <c r="O408" s="378"/>
+      <c r="P408" s="378"/>
+      <c r="Q408" s="378"/>
+      <c r="R408" s="378"/>
+      <c r="S408" s="378"/>
+      <c r="T408" s="378"/>
+      <c r="U408" s="378"/>
+      <c r="V408" s="378"/>
+      <c r="W408" s="378"/>
+      <c r="X408" s="378"/>
+      <c r="Y408" s="378"/>
+      <c r="Z408" s="378"/>
+      <c r="AA408" s="378"/>
+      <c r="AB408" s="378"/>
+      <c r="AC408" s="378"/>
+      <c r="AD408" s="378"/>
+      <c r="AE408" s="378"/>
+      <c r="AF408" s="378"/>
+      <c r="AG408" s="378"/>
+      <c r="AH408" s="378"/>
+      <c r="AI408" s="378"/>
+      <c r="AJ408" s="378"/>
+      <c r="AK408" s="378"/>
+      <c r="AL408" s="378"/>
     </row>
     <row r="409" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A409" s="227" t="s">
@@ -51850,42 +52015,42 @@
       <c r="B409" s="228" t="s">
         <v>49</v>
       </c>
-      <c r="C409" s="370" t="n">
+      <c r="C409" s="379" t="n">
         <v>235</v>
       </c>
-      <c r="F409" s="369"/>
-      <c r="G409" s="369"/>
-      <c r="H409" s="369"/>
-      <c r="I409" s="369"/>
-      <c r="J409" s="369"/>
-      <c r="K409" s="369"/>
-      <c r="L409" s="369"/>
-      <c r="M409" s="369"/>
-      <c r="N409" s="369"/>
-      <c r="O409" s="369"/>
-      <c r="P409" s="369"/>
-      <c r="Q409" s="369"/>
-      <c r="R409" s="369"/>
-      <c r="S409" s="369"/>
-      <c r="T409" s="369"/>
-      <c r="U409" s="369"/>
-      <c r="V409" s="369"/>
-      <c r="W409" s="369"/>
-      <c r="X409" s="369"/>
-      <c r="Y409" s="369"/>
-      <c r="Z409" s="369"/>
-      <c r="AA409" s="369"/>
-      <c r="AB409" s="369"/>
-      <c r="AC409" s="369"/>
-      <c r="AD409" s="369"/>
-      <c r="AE409" s="369"/>
-      <c r="AF409" s="369"/>
-      <c r="AG409" s="369"/>
-      <c r="AH409" s="369"/>
-      <c r="AI409" s="369"/>
-      <c r="AJ409" s="369"/>
-      <c r="AK409" s="369"/>
-      <c r="AL409" s="369"/>
+      <c r="F409" s="378"/>
+      <c r="G409" s="378"/>
+      <c r="H409" s="378"/>
+      <c r="I409" s="378"/>
+      <c r="J409" s="378"/>
+      <c r="K409" s="378"/>
+      <c r="L409" s="378"/>
+      <c r="M409" s="378"/>
+      <c r="N409" s="378"/>
+      <c r="O409" s="378"/>
+      <c r="P409" s="378"/>
+      <c r="Q409" s="378"/>
+      <c r="R409" s="378"/>
+      <c r="S409" s="378"/>
+      <c r="T409" s="378"/>
+      <c r="U409" s="378"/>
+      <c r="V409" s="378"/>
+      <c r="W409" s="378"/>
+      <c r="X409" s="378"/>
+      <c r="Y409" s="378"/>
+      <c r="Z409" s="378"/>
+      <c r="AA409" s="378"/>
+      <c r="AB409" s="378"/>
+      <c r="AC409" s="378"/>
+      <c r="AD409" s="378"/>
+      <c r="AE409" s="378"/>
+      <c r="AF409" s="378"/>
+      <c r="AG409" s="378"/>
+      <c r="AH409" s="378"/>
+      <c r="AI409" s="378"/>
+      <c r="AJ409" s="378"/>
+      <c r="AK409" s="378"/>
+      <c r="AL409" s="378"/>
     </row>
     <row r="410" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A410" s="213" t="s">
@@ -51897,39 +52062,39 @@
       <c r="C410" s="197" t="n">
         <v>0.2</v>
       </c>
-      <c r="F410" s="369"/>
-      <c r="G410" s="369"/>
-      <c r="H410" s="369"/>
-      <c r="I410" s="369"/>
-      <c r="J410" s="369"/>
-      <c r="K410" s="369"/>
-      <c r="L410" s="369"/>
-      <c r="M410" s="369"/>
-      <c r="N410" s="369"/>
-      <c r="O410" s="369"/>
-      <c r="P410" s="369"/>
-      <c r="Q410" s="369"/>
-      <c r="R410" s="369"/>
-      <c r="S410" s="369"/>
-      <c r="T410" s="369"/>
-      <c r="U410" s="369"/>
-      <c r="V410" s="369"/>
-      <c r="W410" s="369"/>
-      <c r="X410" s="369"/>
-      <c r="Y410" s="369"/>
-      <c r="Z410" s="369"/>
-      <c r="AA410" s="369"/>
-      <c r="AB410" s="369"/>
-      <c r="AC410" s="369"/>
-      <c r="AD410" s="369"/>
-      <c r="AE410" s="369"/>
-      <c r="AF410" s="369"/>
-      <c r="AG410" s="369"/>
-      <c r="AH410" s="369"/>
-      <c r="AI410" s="369"/>
-      <c r="AJ410" s="369"/>
-      <c r="AK410" s="369"/>
-      <c r="AL410" s="369"/>
+      <c r="F410" s="378"/>
+      <c r="G410" s="378"/>
+      <c r="H410" s="378"/>
+      <c r="I410" s="378"/>
+      <c r="J410" s="378"/>
+      <c r="K410" s="378"/>
+      <c r="L410" s="378"/>
+      <c r="M410" s="378"/>
+      <c r="N410" s="378"/>
+      <c r="O410" s="378"/>
+      <c r="P410" s="378"/>
+      <c r="Q410" s="378"/>
+      <c r="R410" s="378"/>
+      <c r="S410" s="378"/>
+      <c r="T410" s="378"/>
+      <c r="U410" s="378"/>
+      <c r="V410" s="378"/>
+      <c r="W410" s="378"/>
+      <c r="X410" s="378"/>
+      <c r="Y410" s="378"/>
+      <c r="Z410" s="378"/>
+      <c r="AA410" s="378"/>
+      <c r="AB410" s="378"/>
+      <c r="AC410" s="378"/>
+      <c r="AD410" s="378"/>
+      <c r="AE410" s="378"/>
+      <c r="AF410" s="378"/>
+      <c r="AG410" s="378"/>
+      <c r="AH410" s="378"/>
+      <c r="AI410" s="378"/>
+      <c r="AJ410" s="378"/>
+      <c r="AK410" s="378"/>
+      <c r="AL410" s="378"/>
     </row>
     <row r="411" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A411" s="232" t="s">
@@ -51941,39 +52106,39 @@
       <c r="C411" s="233" t="n">
         <v>2020</v>
       </c>
-      <c r="F411" s="369"/>
-      <c r="G411" s="369"/>
-      <c r="H411" s="369"/>
-      <c r="I411" s="369"/>
-      <c r="J411" s="369"/>
-      <c r="K411" s="369"/>
-      <c r="L411" s="369"/>
-      <c r="M411" s="369"/>
-      <c r="N411" s="369"/>
-      <c r="O411" s="369"/>
-      <c r="P411" s="369"/>
-      <c r="Q411" s="369"/>
-      <c r="R411" s="369"/>
-      <c r="S411" s="369"/>
-      <c r="T411" s="369"/>
-      <c r="U411" s="369"/>
-      <c r="V411" s="369"/>
-      <c r="W411" s="369"/>
-      <c r="X411" s="369"/>
-      <c r="Y411" s="369"/>
-      <c r="Z411" s="369"/>
-      <c r="AA411" s="369"/>
-      <c r="AB411" s="369"/>
-      <c r="AC411" s="369"/>
-      <c r="AD411" s="369"/>
-      <c r="AE411" s="369"/>
-      <c r="AF411" s="369"/>
-      <c r="AG411" s="369"/>
-      <c r="AH411" s="369"/>
-      <c r="AI411" s="369"/>
-      <c r="AJ411" s="369"/>
-      <c r="AK411" s="369"/>
-      <c r="AL411" s="369"/>
+      <c r="F411" s="378"/>
+      <c r="G411" s="378"/>
+      <c r="H411" s="378"/>
+      <c r="I411" s="378"/>
+      <c r="J411" s="378"/>
+      <c r="K411" s="378"/>
+      <c r="L411" s="378"/>
+      <c r="M411" s="378"/>
+      <c r="N411" s="378"/>
+      <c r="O411" s="378"/>
+      <c r="P411" s="378"/>
+      <c r="Q411" s="378"/>
+      <c r="R411" s="378"/>
+      <c r="S411" s="378"/>
+      <c r="T411" s="378"/>
+      <c r="U411" s="378"/>
+      <c r="V411" s="378"/>
+      <c r="W411" s="378"/>
+      <c r="X411" s="378"/>
+      <c r="Y411" s="378"/>
+      <c r="Z411" s="378"/>
+      <c r="AA411" s="378"/>
+      <c r="AB411" s="378"/>
+      <c r="AC411" s="378"/>
+      <c r="AD411" s="378"/>
+      <c r="AE411" s="378"/>
+      <c r="AF411" s="378"/>
+      <c r="AG411" s="378"/>
+      <c r="AH411" s="378"/>
+      <c r="AI411" s="378"/>
+      <c r="AJ411" s="378"/>
+      <c r="AK411" s="378"/>
+      <c r="AL411" s="378"/>
     </row>
     <row r="412" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A412" s="232" t="s">
@@ -51995,7 +52160,7 @@
     </row>
     <row r="415" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A415" s="213" t="s">
-        <v>634</v>
+        <v>636</v>
       </c>
       <c r="B415" s="195" t="s">
         <v>11</v>
@@ -52006,7 +52171,7 @@
     </row>
     <row r="416" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A416" s="213" t="s">
-        <v>635</v>
+        <v>637</v>
       </c>
       <c r="B416" s="195" t="s">
         <v>11</v>
@@ -52017,7 +52182,7 @@
     </row>
     <row r="417" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A417" s="213" t="s">
-        <v>636</v>
+        <v>638</v>
       </c>
       <c r="B417" s="195" t="s">
         <v>11</v>
@@ -52028,12 +52193,12 @@
     </row>
     <row r="418" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A418" s="232" t="s">
-        <v>637</v>
+        <v>639</v>
       </c>
       <c r="B418" s="198" t="s">
         <v>11</v>
       </c>
-      <c r="C418" s="371" t="n">
+      <c r="C418" s="380" t="n">
         <v>0.5</v>
       </c>
     </row>
@@ -52414,16 +52579,16 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="374" t="s">
+      <c r="A1" s="383" t="s">
         <v>107</v>
       </c>
-      <c r="B1" s="375"/>
-      <c r="C1" s="376"/>
-      <c r="E1" s="377"/>
-      <c r="F1" s="378" t="s">
-        <v>638</v>
-      </c>
-      <c r="G1" s="379"/>
+      <c r="B1" s="384"/>
+      <c r="C1" s="385"/>
+      <c r="E1" s="386"/>
+      <c r="F1" s="387" t="s">
+        <v>640</v>
+      </c>
+      <c r="G1" s="388"/>
       <c r="J1" s="212" t="s">
         <v>70</v>
       </c>
@@ -52437,16 +52602,16 @@
       <c r="R1" s="212"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="380" t="s">
+      <c r="A2" s="389" t="s">
         <v>488</v>
       </c>
-      <c r="B2" s="380"/>
-      <c r="C2" s="380"/>
-      <c r="E2" s="377"/>
-      <c r="F2" s="381" t="n">
+      <c r="B2" s="389"/>
+      <c r="C2" s="389"/>
+      <c r="E2" s="386"/>
+      <c r="F2" s="390" t="n">
         <v>2025</v>
       </c>
-      <c r="G2" s="381" t="n">
+      <c r="G2" s="390" t="n">
         <v>2030</v>
       </c>
       <c r="J2" s="213" t="s">
@@ -52455,10 +52620,10 @@
       <c r="K2" s="195" t="s">
         <v>17</v>
       </c>
-      <c r="L2" s="382" t="n">
+      <c r="L2" s="391" t="n">
         <v>2020</v>
       </c>
-      <c r="M2" s="382" t="n">
+      <c r="M2" s="391" t="n">
         <v>2025</v>
       </c>
       <c r="N2" s="214" t="n">
@@ -52478,22 +52643,22 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="383" t="s">
+      <c r="A3" s="392" t="s">
         <v>489</v>
       </c>
-      <c r="B3" s="384" t="s">
-        <v>639</v>
-      </c>
-      <c r="C3" s="385" t="n">
+      <c r="B3" s="393" t="s">
+        <v>641</v>
+      </c>
+      <c r="C3" s="394" t="n">
         <v>0.04</v>
       </c>
-      <c r="E3" s="386" t="s">
-        <v>640</v>
-      </c>
-      <c r="F3" s="387" t="n">
+      <c r="E3" s="395" t="s">
+        <v>642</v>
+      </c>
+      <c r="F3" s="396" t="n">
         <v>0.0371865232692639</v>
       </c>
-      <c r="G3" s="387" t="n">
+      <c r="G3" s="396" t="n">
         <v>0.232670415035861</v>
       </c>
       <c r="J3" s="213" t="s">
@@ -52525,22 +52690,22 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="388" t="s">
+      <c r="A4" s="397" t="s">
         <v>491</v>
       </c>
-      <c r="B4" s="389" t="s">
+      <c r="B4" s="398" t="s">
         <v>17</v>
       </c>
-      <c r="C4" s="390" t="n">
+      <c r="C4" s="399" t="n">
         <v>2025</v>
       </c>
-      <c r="E4" s="386" t="s">
-        <v>641</v>
-      </c>
-      <c r="F4" s="387" t="n">
+      <c r="E4" s="395" t="s">
+        <v>643</v>
+      </c>
+      <c r="F4" s="396" t="n">
         <v>1.6130428775388</v>
       </c>
-      <c r="G4" s="387" t="n">
+      <c r="G4" s="396" t="n">
         <v>0.949592914933259</v>
       </c>
       <c r="J4" s="213" t="s">
@@ -52572,22 +52737,22 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="388" t="s">
+      <c r="A5" s="397" t="s">
         <v>493</v>
       </c>
-      <c r="B5" s="384" t="s">
-        <v>639</v>
-      </c>
-      <c r="C5" s="385" t="n">
+      <c r="B5" s="393" t="s">
+        <v>641</v>
+      </c>
+      <c r="C5" s="394" t="n">
         <v>0.04</v>
       </c>
-      <c r="E5" s="386" t="s">
-        <v>642</v>
-      </c>
-      <c r="F5" s="387" t="n">
+      <c r="E5" s="395" t="s">
+        <v>644</v>
+      </c>
+      <c r="F5" s="396" t="n">
         <v>-0.521132625442432</v>
       </c>
-      <c r="G5" s="387" t="n">
+      <c r="G5" s="396" t="n">
         <v>-0.342735861974531</v>
       </c>
       <c r="J5" s="213" t="s">
@@ -52619,18 +52784,18 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="391" t="s">
+      <c r="A6" s="400" t="s">
         <v>494</v>
       </c>
-      <c r="B6" s="391"/>
-      <c r="C6" s="391"/>
-      <c r="E6" s="386" t="s">
-        <v>643</v>
-      </c>
-      <c r="F6" s="387" t="n">
+      <c r="B6" s="400"/>
+      <c r="C6" s="400"/>
+      <c r="E6" s="395" t="s">
+        <v>645</v>
+      </c>
+      <c r="F6" s="396" t="n">
         <v>-0.00682498781252176</v>
       </c>
-      <c r="G6" s="387" t="n">
+      <c r="G6" s="396" t="n">
         <v>-0.00670819357930043</v>
       </c>
       <c r="J6" s="213" t="s">
@@ -52662,22 +52827,22 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="388" t="s">
+      <c r="A7" s="397" t="s">
         <v>495</v>
       </c>
-      <c r="B7" s="389" t="s">
+      <c r="B7" s="398" t="s">
         <v>17</v>
       </c>
-      <c r="C7" s="392" t="n">
+      <c r="C7" s="401" t="n">
         <v>2020</v>
       </c>
-      <c r="E7" s="386" t="s">
-        <v>644</v>
-      </c>
-      <c r="F7" s="387" t="n">
+      <c r="E7" s="395" t="s">
+        <v>646</v>
+      </c>
+      <c r="F7" s="396" t="n">
         <v>-0.004149377593361</v>
       </c>
-      <c r="G7" s="387" t="n">
+      <c r="G7" s="396" t="n">
         <v>0.825726141078838</v>
       </c>
       <c r="J7" s="213" t="s">
@@ -52709,22 +52874,22 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="393" t="s">
-        <v>645</v>
-      </c>
-      <c r="B8" s="394" t="s">
-        <v>639</v>
-      </c>
-      <c r="C8" s="395" t="n">
+      <c r="A8" s="402" t="s">
+        <v>647</v>
+      </c>
+      <c r="B8" s="403" t="s">
+        <v>641</v>
+      </c>
+      <c r="C8" s="404" t="n">
         <v>0.11</v>
       </c>
-      <c r="E8" s="386" t="s">
-        <v>646</v>
-      </c>
-      <c r="F8" s="387" t="n">
+      <c r="E8" s="395" t="s">
+        <v>648</v>
+      </c>
+      <c r="F8" s="396" t="n">
         <v>-0.375</v>
       </c>
-      <c r="G8" s="387" t="n">
+      <c r="G8" s="396" t="n">
         <v>0</v>
       </c>
       <c r="J8" s="213" t="s">
@@ -52733,10 +52898,10 @@
       <c r="K8" s="195" t="s">
         <v>477</v>
       </c>
-      <c r="L8" s="396" t="n">
+      <c r="L8" s="405" t="n">
         <v>0.000230769</v>
       </c>
-      <c r="M8" s="396" t="n">
+      <c r="M8" s="405" t="n">
         <v>0.000615385</v>
       </c>
       <c r="N8" s="196" t="n">
@@ -52756,22 +52921,22 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="388" t="s">
+      <c r="A9" s="397" t="s">
         <v>497</v>
       </c>
-      <c r="B9" s="384" t="s">
+      <c r="B9" s="393" t="s">
         <v>11</v>
       </c>
-      <c r="C9" s="392" t="n">
+      <c r="C9" s="401" t="n">
         <v>0.25</v>
       </c>
-      <c r="E9" s="386" t="s">
-        <v>647</v>
-      </c>
-      <c r="F9" s="387" t="n">
+      <c r="E9" s="395" t="s">
+        <v>649</v>
+      </c>
+      <c r="F9" s="396" t="n">
         <v>0.238036809815951</v>
       </c>
-      <c r="G9" s="387" t="n">
+      <c r="G9" s="396" t="n">
         <v>0.000710227272727273</v>
       </c>
       <c r="J9" s="213" t="s">
@@ -52803,17 +52968,17 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="397"/>
-      <c r="B10" s="398"/>
-      <c r="C10" s="399"/>
-      <c r="E10" s="386" t="s">
-        <v>648</v>
-      </c>
-      <c r="F10" s="387" t="n">
+      <c r="A10" s="406"/>
+      <c r="B10" s="407"/>
+      <c r="C10" s="408"/>
+      <c r="E10" s="395" t="s">
+        <v>650</v>
+      </c>
+      <c r="F10" s="396" t="n">
         <v>-1</v>
       </c>
-      <c r="G10" s="387" t="s">
-        <v>649</v>
+      <c r="G10" s="396" t="s">
+        <v>651</v>
       </c>
       <c r="J10" s="213" t="s">
         <v>484</v>
@@ -52848,22 +53013,22 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="388" t="s">
+      <c r="A11" s="397" t="s">
         <v>499</v>
       </c>
-      <c r="B11" s="389" t="s">
+      <c r="B11" s="398" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="392" t="n">
+      <c r="C11" s="401" t="n">
         <v>2020</v>
       </c>
-      <c r="E11" s="386" t="s">
-        <v>650</v>
-      </c>
-      <c r="F11" s="387" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="387" t="n">
+      <c r="E11" s="395" t="s">
+        <v>652</v>
+      </c>
+      <c r="F11" s="396" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="396" t="n">
         <v>0</v>
       </c>
       <c r="J11" s="213" t="s">
@@ -52872,7 +53037,7 @@
       <c r="K11" s="195" t="s">
         <v>477</v>
       </c>
-      <c r="L11" s="400" t="n">
+      <c r="L11" s="409" t="n">
         <v>0.000880154</v>
       </c>
       <c r="M11" s="80" t="n">
@@ -52895,22 +53060,22 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="393" t="s">
+      <c r="A12" s="402" t="s">
         <v>500</v>
       </c>
-      <c r="B12" s="394" t="s">
-        <v>639</v>
-      </c>
-      <c r="C12" s="395" t="n">
+      <c r="B12" s="403" t="s">
+        <v>641</v>
+      </c>
+      <c r="C12" s="404" t="n">
         <v>0.04</v>
       </c>
-      <c r="E12" s="386" t="s">
-        <v>651</v>
-      </c>
-      <c r="F12" s="387" t="n">
+      <c r="E12" s="395" t="s">
+        <v>653</v>
+      </c>
+      <c r="F12" s="396" t="n">
         <v>-0.0697461696775669</v>
       </c>
-      <c r="G12" s="387" t="n">
+      <c r="G12" s="396" t="n">
         <v>0.0310626702997275</v>
       </c>
       <c r="J12" s="232" t="s">
@@ -52919,144 +53084,144 @@
       <c r="K12" s="198" t="s">
         <v>305</v>
       </c>
-      <c r="L12" s="401" t="n">
+      <c r="L12" s="410" t="n">
         <v>0.02</v>
       </c>
-      <c r="M12" s="401" t="n">
+      <c r="M12" s="410" t="n">
         <v>0.02</v>
       </c>
-      <c r="N12" s="401" t="n">
+      <c r="N12" s="410" t="n">
         <v>0.02</v>
       </c>
-      <c r="O12" s="401" t="n">
+      <c r="O12" s="410" t="n">
         <v>0.02</v>
       </c>
-      <c r="P12" s="401" t="n">
+      <c r="P12" s="410" t="n">
         <v>0.02</v>
       </c>
-      <c r="Q12" s="401" t="n">
+      <c r="Q12" s="410" t="n">
         <v>0.02</v>
       </c>
-      <c r="R12" s="402" t="n">
+      <c r="R12" s="411" t="n">
         <v>0.02</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="403" t="s">
+      <c r="A13" s="412" t="s">
         <v>121</v>
       </c>
-      <c r="B13" s="403"/>
-      <c r="C13" s="403"/>
-      <c r="E13" s="386" t="s">
-        <v>652</v>
-      </c>
-      <c r="F13" s="387" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="387" t="n">
+      <c r="B13" s="412"/>
+      <c r="C13" s="412"/>
+      <c r="E13" s="395" t="s">
+        <v>654</v>
+      </c>
+      <c r="F13" s="396" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="396" t="n">
         <v>0.00293255131964809</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="404" t="s">
+      <c r="A14" s="413" t="s">
         <v>128</v>
       </c>
-      <c r="B14" s="405" t="s">
-        <v>639</v>
-      </c>
-      <c r="C14" s="406" t="n">
+      <c r="B14" s="414" t="s">
+        <v>641</v>
+      </c>
+      <c r="C14" s="415" t="n">
         <v>0.03</v>
       </c>
-      <c r="E14" s="386" t="s">
-        <v>653</v>
-      </c>
-      <c r="F14" s="387" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="387" t="n">
+      <c r="E14" s="395" t="s">
+        <v>655</v>
+      </c>
+      <c r="F14" s="396" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="396" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="E15" s="386" t="s">
-        <v>654</v>
-      </c>
-      <c r="F15" s="387" t="n">
+      <c r="E15" s="395" t="s">
+        <v>656</v>
+      </c>
+      <c r="F15" s="396" t="n">
         <v>16.656</v>
       </c>
-      <c r="G15" s="387" t="n">
+      <c r="G15" s="396" t="n">
         <v>6.4172</v>
       </c>
-      <c r="L15" s="407" t="n">
+      <c r="L15" s="416" t="n">
         <v>40633</v>
       </c>
-      <c r="M15" s="407" t="n">
+      <c r="M15" s="416" t="n">
         <v>50333</v>
       </c>
-      <c r="N15" s="407" t="n">
+      <c r="N15" s="416" t="n">
         <v>42144</v>
       </c>
-      <c r="O15" s="407" t="n">
+      <c r="O15" s="416" t="n">
         <v>62044</v>
       </c>
-      <c r="P15" s="407" t="n">
+      <c r="P15" s="416" t="n">
         <v>0.0371865232692639</v>
       </c>
-      <c r="Q15" s="407" t="n">
+      <c r="Q15" s="416" t="n">
         <v>0.232670415035861</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="408" t="s">
+      <c r="A16" s="417" t="s">
         <v>122</v>
       </c>
-      <c r="B16" s="409"/>
-      <c r="C16" s="410"/>
-      <c r="L16" s="407" t="n">
+      <c r="B16" s="418"/>
+      <c r="C16" s="419"/>
+      <c r="L16" s="416" t="n">
         <v>21713</v>
       </c>
-      <c r="M16" s="407" t="n">
+      <c r="M16" s="416" t="n">
         <v>39181</v>
       </c>
-      <c r="N16" s="407" t="n">
+      <c r="N16" s="416" t="n">
         <v>56737</v>
       </c>
-      <c r="O16" s="407" t="n">
+      <c r="O16" s="416" t="n">
         <v>76387</v>
       </c>
-      <c r="P16" s="411" t="n">
+      <c r="P16" s="420" t="n">
         <v>16130428775388</v>
       </c>
-      <c r="Q16" s="407" t="n">
+      <c r="Q16" s="416" t="n">
         <v>0.949592914933259</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="412" t="s">
+      <c r="A17" s="421" t="s">
         <v>129</v>
       </c>
-      <c r="B17" s="413" t="s">
-        <v>639</v>
-      </c>
-      <c r="C17" s="414" t="n">
+      <c r="B17" s="422" t="s">
+        <v>641</v>
+      </c>
+      <c r="C17" s="423" t="n">
         <v>0.078</v>
       </c>
-      <c r="L17" s="407" t="n">
+      <c r="L17" s="416" t="n">
         <v>4803</v>
       </c>
-      <c r="M17" s="407" t="n">
+      <c r="M17" s="416" t="n">
         <v>7303</v>
       </c>
-      <c r="N17" s="407" t="n">
+      <c r="N17" s="416" t="n">
         <v>2300</v>
       </c>
-      <c r="O17" s="407" t="n">
+      <c r="O17" s="416" t="n">
         <v>4800</v>
       </c>
-      <c r="P17" s="407" t="n">
+      <c r="P17" s="416" t="n">
         <v>-0.521132625442432</v>
       </c>
-      <c r="Q17" s="407" t="n">
+      <c r="Q17" s="416" t="n">
         <v>-0.342735861974531</v>
       </c>
     </row>
@@ -53064,224 +53229,224 @@
       <c r="A18" s="39"/>
       <c r="B18" s="39"/>
       <c r="C18" s="39"/>
-      <c r="F18" s="415" t="n">
+      <c r="F18" s="424" t="n">
         <v>7156.5</v>
       </c>
       <c r="G18" s="1" t="n">
         <f aca="false">F18*(F4+1)</f>
         <v>18700.2413531064</v>
       </c>
-      <c r="L18" s="407" t="n">
+      <c r="L18" s="416" t="n">
         <v>14359</v>
       </c>
-      <c r="M18" s="407" t="n">
+      <c r="M18" s="416" t="n">
         <v>14609</v>
       </c>
-      <c r="N18" s="407" t="n">
+      <c r="N18" s="416" t="n">
         <v>14261</v>
       </c>
-      <c r="O18" s="407" t="n">
+      <c r="O18" s="416" t="n">
         <v>14511</v>
       </c>
-      <c r="P18" s="407" t="n">
+      <c r="P18" s="416" t="n">
         <v>-0.00682498781252176</v>
       </c>
-      <c r="Q18" s="407" t="n">
+      <c r="Q18" s="416" t="n">
         <v>-0.00670819357930043</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="374" t="s">
+      <c r="A19" s="383" t="s">
         <v>135</v>
       </c>
-      <c r="B19" s="375"/>
-      <c r="C19" s="416"/>
-      <c r="L19" s="407" t="n">
+      <c r="B19" s="384"/>
+      <c r="C19" s="425"/>
+      <c r="L19" s="416" t="n">
         <v>241</v>
       </c>
-      <c r="M19" s="407" t="n">
+      <c r="M19" s="416" t="n">
         <v>241</v>
       </c>
-      <c r="N19" s="407" t="n">
+      <c r="N19" s="416" t="n">
         <v>240</v>
       </c>
-      <c r="O19" s="407" t="n">
+      <c r="O19" s="416" t="n">
         <v>440</v>
       </c>
-      <c r="P19" s="407" t="n">
+      <c r="P19" s="416" t="n">
         <v>-0.004149377593361</v>
       </c>
-      <c r="Q19" s="407" t="n">
+      <c r="Q19" s="416" t="n">
         <v>0.825726141078838</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="417" t="s">
+      <c r="A20" s="426" t="s">
         <v>136</v>
       </c>
-      <c r="B20" s="418" t="s">
+      <c r="B20" s="427" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="419" t="n">
+      <c r="C20" s="428" t="n">
         <v>2017</v>
       </c>
-      <c r="L20" s="407" t="n">
+      <c r="L20" s="416" t="n">
         <v>40</v>
       </c>
-      <c r="M20" s="407" t="n">
+      <c r="M20" s="416" t="n">
         <v>80</v>
       </c>
-      <c r="N20" s="407" t="n">
+      <c r="N20" s="416" t="n">
         <v>25</v>
       </c>
-      <c r="O20" s="407" t="n">
+      <c r="O20" s="416" t="n">
         <v>80</v>
       </c>
-      <c r="P20" s="407" t="n">
+      <c r="P20" s="416" t="n">
         <v>-0.375</v>
       </c>
-      <c r="Q20" s="407" t="n">
+      <c r="Q20" s="416" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="420" t="s">
+      <c r="A21" s="429" t="s">
         <v>138</v>
       </c>
-      <c r="B21" s="421" t="s">
+      <c r="B21" s="430" t="s">
         <v>17</v>
       </c>
-      <c r="C21" s="422" t="n">
+      <c r="C21" s="431" t="n">
         <v>2050</v>
       </c>
-      <c r="L21" s="407" t="n">
+      <c r="L21" s="416" t="n">
         <v>815</v>
       </c>
-      <c r="M21" s="407" t="n">
+      <c r="M21" s="416" t="n">
         <v>1408</v>
       </c>
-      <c r="N21" s="407" t="n">
+      <c r="N21" s="416" t="n">
         <v>1009</v>
       </c>
-      <c r="O21" s="407" t="n">
+      <c r="O21" s="416" t="n">
         <v>1409</v>
       </c>
-      <c r="P21" s="407" t="n">
+      <c r="P21" s="416" t="n">
         <v>0.238036809815951</v>
       </c>
-      <c r="Q21" s="407" t="n">
+      <c r="Q21" s="416" t="n">
         <v>0.000710227272727273</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="420" t="s">
+      <c r="A22" s="429" t="s">
         <v>501</v>
       </c>
-      <c r="B22" s="421" t="s">
-        <v>639</v>
-      </c>
-      <c r="C22" s="423" t="n">
+      <c r="B22" s="430" t="s">
+        <v>641</v>
+      </c>
+      <c r="C22" s="432" t="n">
         <v>0.026</v>
       </c>
-      <c r="L22" s="407" t="n">
+      <c r="L22" s="416" t="n">
         <v>2165</v>
       </c>
-      <c r="M22" s="407" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="407" t="n">
-        <v>0</v>
-      </c>
-      <c r="O22" s="407" t="n">
-        <v>0</v>
-      </c>
-      <c r="P22" s="407" t="n">
+      <c r="M22" s="416" t="n">
+        <v>0</v>
+      </c>
+      <c r="N22" s="416" t="n">
+        <v>0</v>
+      </c>
+      <c r="O22" s="416" t="n">
+        <v>0</v>
+      </c>
+      <c r="P22" s="416" t="n">
         <v>-1</v>
       </c>
-      <c r="Q22" s="407" t="s">
-        <v>649</v>
+      <c r="Q22" s="416" t="s">
+        <v>651</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="388" t="s">
+      <c r="A23" s="397" t="s">
         <v>502</v>
       </c>
-      <c r="B23" s="384" t="s">
-        <v>639</v>
-      </c>
-      <c r="C23" s="424" t="n">
-        <v>0</v>
-      </c>
-      <c r="L23" s="407" t="n">
+      <c r="B23" s="393" t="s">
+        <v>641</v>
+      </c>
+      <c r="C23" s="433" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="416" t="n">
         <v>26612</v>
       </c>
-      <c r="M23" s="407" t="n">
+      <c r="M23" s="416" t="n">
         <v>26612</v>
       </c>
-      <c r="N23" s="407" t="n">
+      <c r="N23" s="416" t="n">
         <v>26612</v>
       </c>
-      <c r="O23" s="407" t="n">
+      <c r="O23" s="416" t="n">
         <v>26612</v>
       </c>
-      <c r="P23" s="407" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="407" t="n">
+      <c r="P23" s="416" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="416" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="388"/>
-      <c r="B24" s="384"/>
-      <c r="C24" s="425" t="s">
+      <c r="A24" s="397"/>
+      <c r="B24" s="393"/>
+      <c r="C24" s="434" t="s">
         <v>305</v>
       </c>
-      <c r="L24" s="407" t="n">
+      <c r="L24" s="416" t="n">
         <v>4373</v>
       </c>
-      <c r="M24" s="407" t="n">
+      <c r="M24" s="416" t="n">
         <v>3670</v>
       </c>
-      <c r="N24" s="407" t="n">
+      <c r="N24" s="416" t="n">
         <v>4068</v>
       </c>
-      <c r="O24" s="407" t="n">
+      <c r="O24" s="416" t="n">
         <v>3784</v>
       </c>
-      <c r="P24" s="407" t="n">
+      <c r="P24" s="416" t="n">
         <v>-0.0697461696775669</v>
       </c>
-      <c r="Q24" s="407" t="n">
+      <c r="Q24" s="416" t="n">
         <v>0.0310626702997275</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="426" t="s">
+      <c r="A25" s="435" t="s">
         <v>503</v>
       </c>
-      <c r="B25" s="427" t="s">
-        <v>639</v>
-      </c>
-      <c r="C25" s="428" t="n">
+      <c r="B25" s="436" t="s">
+        <v>641</v>
+      </c>
+      <c r="C25" s="437" t="n">
         <v>0.012</v>
       </c>
-      <c r="L25" s="407" t="n">
+      <c r="L25" s="416" t="n">
         <v>470</v>
       </c>
-      <c r="M25" s="407" t="n">
+      <c r="M25" s="416" t="n">
         <v>341</v>
       </c>
-      <c r="N25" s="407" t="n">
+      <c r="N25" s="416" t="n">
         <v>470</v>
       </c>
-      <c r="O25" s="407" t="n">
+      <c r="O25" s="416" t="n">
         <v>342</v>
       </c>
-      <c r="P25" s="407" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q25" s="407" t="n">
+      <c r="P25" s="416" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="416" t="n">
         <v>0.00293255131964809</v>
       </c>
     </row>
@@ -53289,150 +53454,150 @@
       <c r="A26" s="39"/>
       <c r="B26" s="39"/>
       <c r="C26" s="39"/>
-      <c r="L26" s="407" t="n">
+      <c r="L26" s="416" t="n">
         <v>7399</v>
       </c>
-      <c r="M26" s="407" t="n">
+      <c r="M26" s="416" t="n">
         <v>3181</v>
       </c>
-      <c r="N26" s="407" t="n">
+      <c r="N26" s="416" t="n">
         <v>7399</v>
       </c>
-      <c r="O26" s="407" t="n">
+      <c r="O26" s="416" t="n">
         <v>3181</v>
       </c>
-      <c r="P26" s="407" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q26" s="407" t="n">
+      <c r="P26" s="416" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="416" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="L27" s="407" t="n">
+      <c r="L27" s="416" t="n">
         <v>500</v>
       </c>
-      <c r="M27" s="407" t="n">
+      <c r="M27" s="416" t="n">
         <v>2500</v>
       </c>
-      <c r="N27" s="407" t="n">
+      <c r="N27" s="416" t="n">
         <v>8828</v>
       </c>
-      <c r="O27" s="407" t="n">
+      <c r="O27" s="416" t="n">
         <v>18543</v>
       </c>
-      <c r="P27" s="411" t="n">
+      <c r="P27" s="420" t="n">
         <v>16656</v>
       </c>
-      <c r="Q27" s="411" t="n">
+      <c r="Q27" s="420" t="n">
         <v>64172</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="16.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C38" s="429" t="n">
+      <c r="C38" s="438" t="n">
         <v>6.5161868524711E-007</v>
       </c>
-      <c r="D38" s="429" t="n">
+      <c r="D38" s="438" t="n">
         <v>5.58035321959433E-007</v>
       </c>
-      <c r="E38" s="429" t="n">
+      <c r="E38" s="438" t="n">
         <v>2.9219735359385E-006</v>
       </c>
-      <c r="F38" s="429" t="n">
+      <c r="F38" s="438" t="n">
         <v>2.04108733475322E-006</v>
       </c>
-      <c r="G38" s="429" t="n">
+      <c r="G38" s="438" t="n">
         <v>4.67798199032692E-007</v>
       </c>
-      <c r="H38" s="429" t="n">
+      <c r="H38" s="438" t="n">
         <v>1.15156800239387E-006</v>
       </c>
-      <c r="I38" s="429" t="n">
+      <c r="I38" s="438" t="n">
         <v>2.78740723393868E-007</v>
       </c>
-      <c r="J38" s="429" t="n">
+      <c r="J38" s="438" t="n">
         <v>5.93179514387632E-007</v>
       </c>
-      <c r="K38" s="429" t="n">
+      <c r="K38" s="438" t="n">
         <v>2.2397859616612E-007</v>
       </c>
-      <c r="L38" s="429" t="n">
+      <c r="L38" s="438" t="n">
         <v>8.94792889409156E-007</v>
       </c>
-      <c r="M38" s="429" t="n">
+      <c r="M38" s="438" t="n">
         <v>3.33816235870076E-007</v>
       </c>
-      <c r="N38" s="429" t="n">
+      <c r="N38" s="438" t="n">
         <v>4.97820658256072E-007</v>
       </c>
-      <c r="O38" s="429" t="n">
+      <c r="O38" s="438" t="n">
         <v>1.55188415866184E-007</v>
       </c>
-      <c r="P38" s="429" t="n">
+      <c r="P38" s="438" t="n">
         <v>2.45947060674221E-007</v>
       </c>
-      <c r="Q38" s="430" t="n">
+      <c r="Q38" s="439" t="n">
         <v>5.39614890128111E-007</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C39" s="431" t="n">
+      <c r="C39" s="440" t="n">
         <f aca="false">C38*1.1</f>
         <v>7.16780553771821E-007</v>
       </c>
-      <c r="D39" s="431" t="n">
+      <c r="D39" s="440" t="n">
         <f aca="false">D38*1.1</f>
         <v>6.13838854155377E-007</v>
       </c>
-      <c r="E39" s="431" t="n">
+      <c r="E39" s="440" t="n">
         <f aca="false">E38*1.1</f>
         <v>3.21417088953235E-006</v>
       </c>
-      <c r="F39" s="431" t="n">
+      <c r="F39" s="440" t="n">
         <f aca="false">F38*1.1</f>
         <v>2.24519606822854E-006</v>
       </c>
-      <c r="G39" s="431" t="n">
+      <c r="G39" s="440" t="n">
         <f aca="false">G38*1.1</f>
         <v>5.14578018935961E-007</v>
       </c>
-      <c r="H39" s="431" t="n">
+      <c r="H39" s="440" t="n">
         <f aca="false">H38*1.1</f>
         <v>1.26672480263326E-006</v>
       </c>
-      <c r="I39" s="431" t="n">
+      <c r="I39" s="440" t="n">
         <f aca="false">I38*1.1</f>
         <v>3.06614795733255E-007</v>
       </c>
-      <c r="J39" s="431" t="n">
+      <c r="J39" s="440" t="n">
         <f aca="false">J38*1.1</f>
         <v>6.52497465826395E-007</v>
       </c>
-      <c r="K39" s="431" t="n">
+      <c r="K39" s="440" t="n">
         <f aca="false">K38*1.1</f>
         <v>2.46376455782732E-007</v>
       </c>
-      <c r="L39" s="431" t="n">
+      <c r="L39" s="440" t="n">
         <f aca="false">L38*1.1</f>
         <v>9.84272178350072E-007</v>
       </c>
-      <c r="M39" s="431" t="n">
+      <c r="M39" s="440" t="n">
         <f aca="false">M38*1.1</f>
         <v>3.67197859457083E-007</v>
       </c>
-      <c r="N39" s="431" t="n">
+      <c r="N39" s="440" t="n">
         <f aca="false">N38*1.1</f>
         <v>5.4760272408168E-007</v>
       </c>
-      <c r="O39" s="431" t="n">
+      <c r="O39" s="440" t="n">
         <f aca="false">O38*1.1</f>
         <v>1.70707257452802E-007</v>
       </c>
-      <c r="P39" s="431" t="n">
+      <c r="P39" s="440" t="n">
         <f aca="false">P38*1.1</f>
         <v>2.70541766741643E-007</v>
       </c>
-      <c r="Q39" s="431" t="n">
+      <c r="Q39" s="440" t="n">
         <f aca="false">Q38*1.1</f>
         <v>5.93576379140922E-007</v>
       </c>

</xml_diff>